<commit_message>
Update order ledger with first recorded production job
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/skills/robot-ross/orders.xlsx
+++ b/skills/robot-ross/orders.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -483,6 +483,38 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-02-19 14:33:56</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>write</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Im a movie star</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2026-02-19 14:35:35</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>/Users/miguelrodriguez/Movies/2026-02-19 14-33-56.mov</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add get_last_video_url() to order_log for artist_poller proof-of-work callback
Reads the last non-empty Video URL from orders.xlsx so artist_poller
can include it in the complete() call back to Salesman.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/skills/robot-ross/orders.xlsx
+++ b/skills/robot-ross/orders.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -515,6 +515,708 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-02-19 17:16:49</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>write</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>happy
+birthday
+Cynthia</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2026-02-19 17:19:17</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>/Users/miguelrodriguez/Movies/2026-02-19 17-16-49.mov</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-02-19 22:17:00</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>write</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Happy
+Birthday
+Cynthia
+.</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2026-02-19 22:19:31</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>/Users/miguelrodriguez/Movies/2026-02-19 22-17-00.mov</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-02-19 22:20:05</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>write</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Happy
+Birthday
+Cynthia
+.</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2026-02-19 22:22:18</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>/Users/miguelrodriguez/Movies/2026-02-19 22-20-05.mov</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-02-19 22:33:13</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>svg</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>donkey.svg</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>in_progress</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-02-19 22:41:03</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>svg</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>donkey.svg</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>in_progress</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-02-19 22:48:48</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>svg</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>donkey.svg</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>in_progress</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-02-20 13:45:55</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>miguel+test@bigbearengineering.com</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>write</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Greetings from Sales</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>in_progress</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-02-20 13:53:25</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>shopify-order-1002</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>write</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Greetings from Sales</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>2026-02-20 13:55:37</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=nGc70czngZk</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-02-23 11:29:14</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>svg</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>bunny.svg</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>in_progress</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-02-23 11:31:38</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>svg</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>bunny.svg</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>in_progress</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-02-23 11:35:03</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>svg</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>bunny.svg</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>2026-02-23 11:38:08</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=MbEKYv3zCOQ</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-02-23 12:05:15</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>svg</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>/Users/miguelrodriguez/Downloads/Bunny.svg</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>2026-02-23 12:08:20</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=ob69UrbqQIA</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-02-24 17:57:00</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>John</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>write</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Shopify order 820982911946154500</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>in_progress</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-02-24 18:01:09</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Rodriguez</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>write</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Shopify order 7439027110225</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>2026-02-24 18:03:26</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=jRQQUxaD3h0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-02-25 14:45:12</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Miguel</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>write</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Shopify order 7440630546769</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>2026-02-25 14:47:59</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=bq9jMtgJC4A</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-02-25 14:57:27</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Miguel</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>write</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Shopify order 7440676061521</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>2026-02-25 15:00:12</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=geV66AkEA3U</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-02-25 16:19:39</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Miguel</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>write</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Shopify order 7440834494801</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>2026-02-25 16:22:32</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=qzVWjsUHGlU</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-02-25 16:25:43</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Miguel</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>write</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Shopify order 7440842162513</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>2026-02-25 16:28:01</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=jl1pacZYdic</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-02-25 17:02:48</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Miguel</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>write</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Shopify order 7440915890513</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>2026-02-25 17:05:36</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=jbvHctvfEQk</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-02-25 17:18:13</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Miguel</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>write</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>a teddy and a bunny</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>2026-02-25 17:20:04</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=GuMlCxCTGyM</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-02-25 17:29:32</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Miguel</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>svg</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Draw a Bunny and a Bear</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>2026-02-25 17:30:40</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>failed</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=Bh6Gg-otujU</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-02-25 17:40:18</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Miguel</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>sketch</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Draw me a bunny and a bear</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>2026-02-25 17:42:26</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=lQludLHn_Og</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: merge Mexico-era features from bobrossskill into robot-ross
</commit_message>
<xml_diff>
--- a/skills/robot-ross/orders.xlsx
+++ b/skills/robot-ross/orders.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I24"/>
+  <dimension ref="A1:I45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1217,6 +1217,743 @@
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-02-25 19:34:03</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Miguel</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>write</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Shopify order 7441203003729</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>2026-02-25 19:36:19</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=ucc38Y514Ik</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-02-26 15:15:31</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>RobotRoss_Demo</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>write</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>A cute bunny and a friendly bear\nsitting together under a tree</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>2026-02-26 15:19:07</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=cmXL2PpYpU4</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-02-26 15:46:05</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Gemini_Bot</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>write</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Property of Gemini</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>2026-02-26 15:48:08</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=KEPE-7kpspo</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-02-26 15:51:19</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Gemini_Bot</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>write</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Property of Gemini</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>2026-02-26 15:53:24</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=Cb7-GDXr_Ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-02-26 21:58:15</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>tester_gemini</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>write</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Hello Virtuals! Integration Test</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>2026-02-26 22:00:47</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=frP1rdQGmVY</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-02-27 10:36:05</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Miguel</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>sketch</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>A poodle dog</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>2026-02-27 10:37:34</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-02-27 11:22:02</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Miguel</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>sketch</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Poodle dog</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>2026-02-27 11:23:55</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=H8jM9f7qP1w</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-02-27 11:46:16</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Miguel</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>sketch</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>A golden rocket ship launching from a field of happy little trees.</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>2026-02-27 11:47:39</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=JEAgMUHvLzM</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-02-27 12:09:58</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Miguel</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>sketch</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>A happy little bird</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>2026-02-27 12:11:37</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=xqDWV77CXDo</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-02-27 13:15:35</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Mimi</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>write</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>I love your bum bum!!!</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>2026-02-27 13:17:50</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=iZTemSt84wk</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-02-27 13:33:40</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>tester_gemini</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>write</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Hello Virtuals! Integration Test</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>2026-02-27 13:36:13</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=l5_le0FSnYY</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-02-27 13:39:35</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Enrique</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>sketch</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Draw the Earth globe, showing continental contours: Europe, parts of Africa and Asia, etc.</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>2026-02-27 13:41:18</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=aFTRMryI7ZM</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-02-27 13:53:37</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Miguel</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>sketch</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>A happy little bird</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>2026-02-27 13:56:07</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=ZubC3H6TMSs</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-02-27 13:56:19</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Enrique</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>sketch</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Draw the Earth globe, showing continental contours: Europe, parts of Africa and Asia</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>2026-02-27 13:58:42</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=yMJu-RArHWw</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-03-01 08:44:04</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>sketch</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>A teddy bear and a bunny sitting side by side watching the sunset</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>2026-03-01 08:45:05</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>failed</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=mONI28uXYaw</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-03-01 08:47:25</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>sketch</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>A teddy bear and a bunny sitting side by side watching the sunset</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>in_progress</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-03-01 08:51:46</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>sketch</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>A teddy bear and a bunny sitting side by side watching the sunset</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>2026-03-01 08:57:49</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=YiRf_vypfSA</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-03-01 19:29:55</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Miguel</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>sketch</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>cuckoo clock</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>2026-03-01 19:33:28</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=Gwie7k-Ps4o</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-03-02 07:47:08</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Miguel</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>sketch</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>cuckoo clock</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>2026-03-02 07:49:56</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=uzh76pkP0Jw</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-03-07 11:14:51</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>testclient</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>write</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>a happy little tree</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>2026-03-07 11:17:04</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-03-09 19:40:54</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>testclient</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>sketch</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>a happy little tree</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>2026-03-09 19:43:25</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>success</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>